<commit_message>
Fix of test cases
</commit_message>
<xml_diff>
--- a/1-Manual Test Plans/ParadoxQATest_WebTestPlan_DarioSC.xlsx
+++ b/1-Manual Test Plans/ParadoxQATest_WebTestPlan_DarioSC.xlsx
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dario\Documents\GitHub\ParadoxQATest_DarioSC\1-Manual Test Plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8C6C770-6ABA-476E-80F3-05E7BC3C59EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEF76420-520E-4168-88CC-4CCAF850C21C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestPlan-NoLogIn" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TestPlan-NoLogIn'!$A$1:$J$1</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -66,6 +63,17 @@
     <t>High</t>
   </si>
   <si>
+    <t>Because this is the first page users will see on the company's website, and it showcases the most important project currently being promoted.</t>
+  </si>
+  <si>
+    <t>&gt; No user is logged in 
+&gt; No games in the cart</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/discover]
+2.- Click the [AVAILABLE NOW &gt;] button</t>
+  </si>
+  <si>
     <t>2.1.- The announced game's website should open, changing the header from the Paradox banner to the game banner
 2.2.- The hero section containing the loop video will stay in the same place
 2.3.- The [AVAILABLE NOW &gt;] button should change to [BUY NOW 🛒]</t>
@@ -78,188 +86,6 @@
   </si>
   <si>
     <t>Cookie settings test</t>
-  </si>
-  <si>
-    <t>Discover_03</t>
-  </si>
-  <si>
-    <t>Current language test</t>
-  </si>
-  <si>
-    <t>Mid</t>
-  </si>
-  <si>
-    <t>2. &amp; 4.- A drop-down menu will appear displaying all the languages supported by the website
-3.- Simplified Chinese will be applied to the website, and a pop-up will appear warning that it is in beta
-5.- The website will return to the selected language</t>
-  </si>
-  <si>
-    <t>Discover_04</t>
-  </si>
-  <si>
-    <t>Responsive test</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/discover]
-2.- Position the device in portrait mode and scroll down in the Discover page
-3.- Position the device in landscape mode and scroll down in the Discover page</t>
-  </si>
-  <si>
-    <t>2. &amp; 3.- The website content should display and scale properly, with no text, images, or loop videos cut off</t>
-  </si>
-  <si>
-    <t>Fail</t>
-  </si>
-  <si>
-    <t>RP-1310261</t>
-  </si>
-  <si>
-    <t>Discover_05</t>
-  </si>
-  <si>
-    <t>Back to top button</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>Because it is not a fundamental feature of the website</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/discover]
-2.- Scroll down for a while
-3.- Click on the button [↑]</t>
-  </si>
-  <si>
-    <t>2.- The "Go up" button [↑] will appear in the bottom-right corner
-3.- The website will return to the top of the page</t>
-  </si>
-  <si>
-    <t>AllGames_01</t>
-  </si>
-  <si>
-    <t>Search bar test</t>
-  </si>
-  <si>
-    <t>2.- The "No matching games" message will appear, with no games displayed
-3.- The text just inserted in the [SEARCH] bar will be deleted
-4.- All games related to that title will be displayed
-5.- A pop-up should confirm that the game has been added to the cart, and the [🛒] button will show the number of games added</t>
-  </si>
-  <si>
-    <t>AllGames_02</t>
-  </si>
-  <si>
-    <t>Choose edition test</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
-2.- Find a game that gives the option of [CHOOSE EDITION] and click on it
-3.- Add to cart the regular edition of the game
-4.- Open [https://www.paradoxinteractive.com/our-games/all-games]
-5.- Search for the same game and click again on [CHOOSE EDITION] to pick another edition</t>
-  </si>
-  <si>
-    <t>RP-1310262</t>
-  </si>
-  <si>
-    <t>AllGames_03</t>
-  </si>
-  <si>
-    <t>Essential filters test</t>
-  </si>
-  <si>
-    <t>2. &amp; 3.- The games will be displayed according to the selected filters</t>
-  </si>
-  <si>
-    <t>AllGames_04</t>
-  </si>
-  <si>
-    <t>Personalized filters test</t>
-  </si>
-  <si>
-    <t>2.- The games will be displayed according to the selected filters
-3.- All current filters will be cleared, and the games will return to the unfiltered display</t>
-  </si>
-  <si>
-    <t>AllGames_05</t>
-  </si>
-  <si>
-    <t>Added to cart test</t>
-  </si>
-  <si>
-    <t>2.- A pop-up should confirm that the game has been added to the cart, and the [🛒] button will show the number of games added
-3.- The [Add to cart] button will change to [Added to cart], become disabled, and have a different hover behavior</t>
-  </si>
-  <si>
-    <t>AllGames_06</t>
-  </si>
-  <si>
-    <t>Go to on sale test</t>
-  </si>
-  <si>
-    <t>2. &amp; 4.- The On Sale site will open</t>
-  </si>
-  <si>
-    <t>OnSale_01</t>
-  </si>
-  <si>
-    <t>On sale tag display test</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/on-sale]
-2.- Review all the games on the On Sale site</t>
-  </si>
-  <si>
-    <t>YourCart_01</t>
-  </si>
-  <si>
-    <t>YourCart_02</t>
-  </si>
-  <si>
-    <t>Saving cart test</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
-2.- Add one or more games to cart
-3.- Close the browser window and open [https://www.paradoxinteractive.com/our-games/cart]
-4.- Close the browser completely 
-5.- Open the closed browser and go to: [https://www.paradoxinteractive.com/our-games/cart]</t>
-  </si>
-  <si>
-    <t>2.- The games will be added to the cart normally. A pop-up will confirm each game as it is added
-3. &amp; 5.- The cart page will open with the latest saved information</t>
-  </si>
-  <si>
-    <t>YourCart_03</t>
-  </si>
-  <si>
-    <t>Promo codes test</t>
-  </si>
-  <si>
-    <t>2.- The games will be added to the cart normally. A pop-up will confirm each game as it is added
-4.- The [ADD PROMO CODE] button will appear below the text frame
-     4.1.- A warning pop-up should appear next to the text frame
-     4.2.- The text frame will turn bold and red, and the message "Voucher has to be at least 8 characters long." will appear below it
-     4.3.- The entered code will disappear, and an error pop-up will appear in the bottom-right corner
-     4.4.- The discount will be applied, the summary will be updated with the discount information, and a confirmation pop-up will appear in the bottom-right corner</t>
-  </si>
-  <si>
-    <t>YourCart_04</t>
-  </si>
-  <si>
-    <t>Back to All Games</t>
-  </si>
-  <si>
-    <t>Because this is the first page users will see on the company's website, and it showcases the most important project currently being promoted.</t>
-  </si>
-  <si>
-    <t>&gt; No user is logged in 
-&gt; No games in the cart</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/discover]
-2.- Click the [AVAILABLE NOW &gt;] button</t>
   </si>
   <si>
     <t>Because cookie consent is a fundamental legal requirement for users.</t>
@@ -269,170 +95,6 @@
 private browsing for this test
 &gt; No user is logged in 
 &gt; No games in the cart</t>
-  </si>
-  <si>
-    <t>1.- The Discover Paradox website will open, and a "Cookies and targeting" pop-up will appear
-     1.1.- The Cookie settings sidebar will open
-     1.2. &amp; 1.3.- The windows will disappear, and the cookies will be set according to the selected option
-2.- A sidebar will open showing the current cookie settings
-     2.1. &amp; 2.2. &amp; 2.3. &amp; 2.4.- The toggles will function normally; when all three are off, the [Allow All] button will appear
-     2.5.- All toggles will switch on, and the sidebar will close
-3.- The sidebar will disappear, returning to the Discover site
-     3.1.- The sidebar will disappear with the toggles switched off
-     3.2.- The current toggle selection will be saved and the sidebar will close
-     3.3.- The sidebar will close without saving any changes</t>
-  </si>
-  <si>
-    <t>AUTOMATION CANDIDATE: This test is very important, both from a legal perspective and because of how the company collects user data. For that reason, verifying that it works correctly at all times is valuable. Also, because this is a longer test, automating it reduces the risk of human error.</t>
-  </si>
-  <si>
-    <t>Because only one language is currently fully available. If more languages become available, this test's priority will increase.</t>
-  </si>
-  <si>
-    <t>&gt; Refresh or reopen the website
-&gt; No user is logged in 
-&gt; No games in the cart</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/discover]
-2.- Open the language drop-down menu by clicking [🌐 ENGLISH] in the header
-3.- Click [中文（简体)]
-4.- Open the language drop-down menu by clicking [🌐 中文（简体)] in the header
-5.- Click [ENGLISH]</t>
-  </si>
-  <si>
-    <t>&gt; This test requires a smartphone or a tablet
-&gt; No user is logged in 
-&gt; No games in the cart</t>
-  </si>
-  <si>
-    <t>&gt; The website needs to be at the top of the page
-&gt; No user is logged in 
-&gt; No games in the cart</t>
-  </si>
-  <si>
-    <t>Because it is a common feature used to search for games easily.</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
-2.- Click into the [SEARCH] bar and write the name of a non-Paradox game (repeat this step five times with non-Paradox games)
-3.- Click the [X] and [CLEAR ALL (X)] buttons in the [SEARCH] bar
-4.- Click into the [SEARCH] bar and write the name of a Paradox game (repeat this step five times with Paradox games)
-5.- Add all the searched games to the cart</t>
-  </si>
-  <si>
-    <t>This test has been automated because we can run as many searches as there are games in the test. In other words, we can check names one by one automatically, allowing a tester to focus on issues that affect the user experience.</t>
-  </si>
-  <si>
-    <t>Because it is how users access each game's specific store.</t>
-  </si>
-  <si>
-    <t>2. &amp; 5.- The game's page should open and display its different editions. In step 5, the previously selected edition should be marked [ADDED TO CART].
-3.- The selected edition will be added to the cart.</t>
-  </si>
-  <si>
-    <t>Because users will choose these filters to search among the different types of games in the store.</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
-2.- Open the [Ordering filter] drop-down menu and select each option one by one
-3.- Click each of the main filters displayed below the [SEARCH] bar</t>
-  </si>
-  <si>
-    <t>Because users will use the search bar and essential filters before using personalized filters.</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
-2.- Open the [FILTER] drop-down menu and select each button one by one
-3.- Scroll to the top of the page and click [CLEAR ALL (X)]</t>
-  </si>
-  <si>
-    <t>AUTOMATED TEST: Like AllGames_01, this test is automated because checking the website's filters one by one could lead to human error. Also, since we do not know how much the site may grow in the future, it is better to keep this test automated.</t>
-  </si>
-  <si>
-    <t>Because this is the necessary confirmation to let users know they can proceed to checkout with their purchase.</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
-2.- Add any game to the cart by clicking [Add to Cart]
-3.- Hover over the [Add to Cart] button for the game just added</t>
-  </si>
-  <si>
-    <t>Because it is a somewhat hidden feature at the bottom of the All Games page, where it serves as a promotional hook.</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
-2.- Scroll to the end of the game list and click the image with the red "ON SALE" text
-3.- Open [https://www.paradoxinteractive.com/our-games/all-games]
-4.- Scroll to the end of the game list and click [SHOP SALE NOW]</t>
-  </si>
-  <si>
-    <t>Because it is important that all games shown in the sale section actually display the sale tag.</t>
-  </si>
-  <si>
-    <t>2.- The games should display their sale tags in the upper-left corner of each card, showing the discount.</t>
-  </si>
-  <si>
-    <t>Essential cart functions test</t>
-  </si>
-  <si>
-    <t>Because these are the most essential features of the website's purchasing system.</t>
-  </si>
-  <si>
-    <t>2. &amp; 4.- A pop-up should confirm that the games have been added to the cart, and the [🛒] button will show the number of games added
-5.- The cart page will open, displaying the selected games and the purchase summary with the sale price applied
-6.- The cart will update automatically to show the number of games and the purchase summary</t>
-  </si>
-  <si>
-    <t>AUTOMATED TEST: This test is essential to the operation of any store. It should run regularly so that, if it fails, we can determine whether the website is down. This test is important before launching a new product, but it does not simulate the request volume needed to determine whether the site can handle high traffic.</t>
-  </si>
-  <si>
-    <t>Because this system makes it easier for users to complete their purchases.</t>
-  </si>
-  <si>
-    <t>AUTOMATED TEST: This is another essential feature that should be checked regularly to determine whether the website is down or whether a code change has broken this flow. I would extend this test to cover payment methods, but that is outside the scope of the assignment.</t>
-  </si>
-  <si>
-    <t>Because not all users have discount codes. I could raise this case's priority to High during promotional periods when many promo codes are issued.</t>
-  </si>
-  <si>
-    <t>&gt; A promo code is needed for QA testing
-&gt; No user is logged in 
-&gt; No games in the cart</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
-2.- Add one game to the cart
-3.- Open the cart by clicking the [🛒] button
-4.- Below the summary, click the input field with the placeholder text "Do you have a promo code?"
-     4.1.- Leave the field empty and click [ADD PROMO CODE]
-     4.2.- Enter 3 random characters and click [ADD PROMO CODE]
-     4.3.- Enter 8 random characters and click [ADD PROMO CODE]
-     4.4.- Enter the QA promo code and click [ADD PROMO CODE]</t>
-  </si>
-  <si>
-    <t>Because the website header already has an [ALL GAMES] button that is always visible.</t>
-  </si>
-  <si>
-    <t>&gt; No user is logged in</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/cart]
-2.- Click [GO TO ALL GAMES]
-3.- Open [https://www.paradoxinteractive.com/our-games/cart]
-4.- Click [← CONTINUE SHOPPING]</t>
-  </si>
-  <si>
-    <t>1. &amp; 3.- The cart page should open. Since the cart is empty, the empty-cart state should be displayed.
-2. &amp; 4.- The All Games page should open.</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
-2.- Add one game to the cart
-3.- Open [https://www.paradoxinteractive.com/our-games/on-sale]
-4.- Add one game on sale to the cart
-5.- Open the cart by clicking the [🛒] button and check the summary
-6.- Remove the game on sale and check the summary</t>
   </si>
   <si>
     <r>
@@ -472,6 +134,348 @@
      3.2.- Click [Confirm My Choices]
      3.3.- Click the [X] button in the upper-right corner</t>
     </r>
+  </si>
+  <si>
+    <t>1.- The Discover Paradox website will open, and a "Cookies and targeting" pop-up will appear
+     1.1.- The Cookie settings sidebar will open
+     1.2. &amp; 1.3.- The windows will disappear, and the cookies will be set according to the selected option
+2.- A sidebar will open showing the current cookie settings
+     2.1. &amp; 2.2. &amp; 2.3. &amp; 2.4.- The toggles will function normally; when all three are off, the [Allow All] button will appear
+     2.5.- All toggles will switch on, and the sidebar will close
+3.- The sidebar will disappear, returning to the Discover site
+     3.1.- The sidebar will disappear with the toggles switched off
+     3.2.- The current toggle selection will be saved and the sidebar will close
+     3.3.- The sidebar will close without saving any changes</t>
+  </si>
+  <si>
+    <t>AUTOMATION CANDIDATE: This test is very important, both from a legal perspective and because of how the company collects user data. For that reason, verifying that it works correctly at all times is valuable. Also, because this is a longer test, automating it reduces the risk of human error.</t>
+  </si>
+  <si>
+    <t>Discover_03</t>
+  </si>
+  <si>
+    <t>Current language test</t>
+  </si>
+  <si>
+    <t>Mid</t>
+  </si>
+  <si>
+    <t>Because only one language is currently fully available. If more languages become available, this test's priority will increase.</t>
+  </si>
+  <si>
+    <t>&gt; Refresh or reopen the website
+&gt; No user is logged in 
+&gt; No games in the cart</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/discover]
+2.- Open the language drop-down menu by clicking [🌐 ENGLISH] in the header
+3.- Click [中文（简体)]
+4.- Open the language drop-down menu by clicking [🌐 中文（简体)] in the header
+5.- Click [ENGLISH]</t>
+  </si>
+  <si>
+    <t>2. &amp; 4.- A drop-down menu will appear displaying all the languages supported by the website
+3.- Simplified Chinese will be applied to the website, and a pop-up will appear warning that it is in beta
+5.- The website will return to the selected language</t>
+  </si>
+  <si>
+    <t>Discover_04</t>
+  </si>
+  <si>
+    <t>Responsive test</t>
+  </si>
+  <si>
+    <t>&gt; This test requires a smartphone or a tablet
+&gt; No user is logged in 
+&gt; No games in the cart</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/discover]
+2.- Position the device in portrait mode and scroll down in the Discover page
+3.- Position the device in landscape mode and scroll down in the Discover page</t>
+  </si>
+  <si>
+    <t>2. &amp; 3.- The website content should display and scale properly, with no text, images, or loop videos cut off</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>RP-1310261</t>
+  </si>
+  <si>
+    <t>Discover_05</t>
+  </si>
+  <si>
+    <t>Back to top button</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Because it is not a fundamental feature of the website</t>
+  </si>
+  <si>
+    <t>&gt; The website needs to be at the top of the page
+&gt; No user is logged in 
+&gt; No games in the cart</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/discover]
+2.- Scroll down for a while
+3.- Click on the button [↑]</t>
+  </si>
+  <si>
+    <t>2.- The "Go up" button [↑] will appear in the bottom-right corner
+3.- The website will return to the top of the page</t>
+  </si>
+  <si>
+    <t>AllGames_01</t>
+  </si>
+  <si>
+    <t>Search bar test</t>
+  </si>
+  <si>
+    <t>Because it is a common feature used to search for games easily.</t>
+  </si>
+  <si>
+    <t>2.- The "No matching games" message will appear, with no games displayed
+3.- The text just inserted in the [SEARCH] bar will be deleted
+4.- All games related to that title will be displayed
+5.- A pop-up should confirm that the game has been added to the cart, and the [🛒] button will show the number of games added</t>
+  </si>
+  <si>
+    <t>This test has been automated because we can run as many searches as there are games in the test. In other words, we can check names one by one automatically, allowing a tester to focus on issues that affect the user experience.</t>
+  </si>
+  <si>
+    <t>AllGames_02</t>
+  </si>
+  <si>
+    <t>Choose edition test</t>
+  </si>
+  <si>
+    <t>2. &amp; 5.- The game's page should open and display its different editions. In step 5, the previously selected edition should be marked [ADDED TO CART].
+3.- The selected edition will be added to the cart.</t>
+  </si>
+  <si>
+    <t>RP-1310262</t>
+  </si>
+  <si>
+    <t>AllGames_03</t>
+  </si>
+  <si>
+    <t>Essential filters test</t>
+  </si>
+  <si>
+    <t>Because users will choose these filters to search among the different types of games in the store.</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
+2.- Open the [Ordering filter] drop-down menu and select each option one by one
+3.- Click each of the main filters displayed below the [SEARCH] bar</t>
+  </si>
+  <si>
+    <t>2. &amp; 3.- The games will be displayed according to the selected filters</t>
+  </si>
+  <si>
+    <t>AllGames_04</t>
+  </si>
+  <si>
+    <t>Personalized filters test</t>
+  </si>
+  <si>
+    <t>Because users will use the search bar and essential filters before using personalized filters.</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
+2.- Open the [FILTER] drop-down menu and select each button one by one
+3.- Scroll to the top of the page and click [CLEAR ALL (X)]</t>
+  </si>
+  <si>
+    <t>2.- The games will be displayed according to the selected filters
+3.- All current filters will be cleared, and the games will return to the unfiltered display</t>
+  </si>
+  <si>
+    <t>AUTOMATED TEST: Like AllGames_01, this test is automated because checking the website's filters one by one could lead to human error. Also, since we do not know how much the site may grow in the future, it is better to keep this test automated.</t>
+  </si>
+  <si>
+    <t>AllGames_05</t>
+  </si>
+  <si>
+    <t>Added to cart test</t>
+  </si>
+  <si>
+    <t>Because this is the necessary confirmation to let users know they can proceed to checkout with their purchase.</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
+2.- Add any game to the cart by clicking [Add to Cart]
+3.- Hover over the [Add to Cart] button for the game just added</t>
+  </si>
+  <si>
+    <t>2.- A pop-up should confirm that the game has been added to the cart, and the [🛒] button will show the number of games added
+3.- The [Add to cart] button will change to [Added to cart], become disabled, and have a different hover behavior</t>
+  </si>
+  <si>
+    <t>AllGames_06</t>
+  </si>
+  <si>
+    <t>Because it is a somewhat hidden feature at the bottom of the All Games page, where it serves as a promotional hook.</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
+2.- Scroll to the end of the game list and click the image with the red "ON SALE" text
+3.- Open [https://www.paradoxinteractive.com/our-games/all-games]
+4.- Scroll to the end of the game list and click [SHOP SALE NOW]</t>
+  </si>
+  <si>
+    <t>OnSale_01</t>
+  </si>
+  <si>
+    <t>On sale tag display test</t>
+  </si>
+  <si>
+    <t>Because it is important that all games shown in the sale section actually display the sale tag.</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/on-sale]
+2.- Review all the games on the On Sale site</t>
+  </si>
+  <si>
+    <t>YourCart_01</t>
+  </si>
+  <si>
+    <t>Essential cart functions test</t>
+  </si>
+  <si>
+    <t>Because these are the most essential features of the website's purchasing system.</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
+2.- Add one game to the cart
+3.- Open [https://www.paradoxinteractive.com/our-games/on-sale]
+4.- Add one game on sale to the cart
+5.- Open the cart by clicking the [🛒] button and check the summary
+6.- Remove the game on sale and check the summary</t>
+  </si>
+  <si>
+    <t>2. &amp; 4.- A pop-up should confirm that the games have been added to the cart, and the [🛒] button will show the number of games added
+5.- The cart page will open, displaying the selected games and the purchase summary with the sale price applied
+6.- The cart will update automatically to show the number of games and the purchase summary</t>
+  </si>
+  <si>
+    <t>AUTOMATED TEST: This test is essential to the operation of any store. It should run regularly so that, if it fails, we can determine whether the website is down. This test is important before launching a new product, but it does not simulate the request volume needed to determine whether the site can handle high traffic.</t>
+  </si>
+  <si>
+    <t>YourCart_02</t>
+  </si>
+  <si>
+    <t>Because this system makes it easier for users to complete their purchases.</t>
+  </si>
+  <si>
+    <t>AUTOMATED TEST: This is another essential feature that should be checked regularly to determine whether the website is down or whether a code change has broken this flow. I would extend this test to cover payment methods, but that is outside the scope of the assignment.</t>
+  </si>
+  <si>
+    <t>YourCart_03</t>
+  </si>
+  <si>
+    <t>Promo codes test</t>
+  </si>
+  <si>
+    <t>Because not all users have discount codes. I could raise this case's priority to High during promotional periods when many promo codes are issued.</t>
+  </si>
+  <si>
+    <t>&gt; A promo code is needed for QA testing
+&gt; No user is logged in 
+&gt; No games in the cart</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
+2.- Add one game to the cart
+3.- Open the cart by clicking the [🛒] button
+4.- Below the summary, click the input field with the placeholder text "Do you have a promo code?"
+     4.1.- Leave the field empty and click [ADD PROMO CODE]
+     4.2.- Enter 3 random characters and click [ADD PROMO CODE]
+     4.3.- Enter 8 random characters and click [ADD PROMO CODE]
+     4.4.- Enter the QA promo code and click [ADD PROMO CODE]</t>
+  </si>
+  <si>
+    <t>YourCart_04</t>
+  </si>
+  <si>
+    <t>Back to All Games</t>
+  </si>
+  <si>
+    <t>Because the website header already has an [ALL GAMES] button that is always visible.</t>
+  </si>
+  <si>
+    <t>&gt; No user is logged in
+&gt; No games in the cart</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
+2.- Click the [SEARCH] bar and enter the name of a non-Paradox game (repeat this step five times with different non-Paradox games)
+3.- Click the [X] and [CLEAR ALL (X)] buttons in the [SEARCH] bar
+4.- Click the [SEARCH] bar and enter the name of a Paradox game (repeat this step five times with different Paradox games)
+5.- Add all the searched games to the cart</t>
+  </si>
+  <si>
+    <t>Because this is how users access each game's store page.</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
+2.- Find a game that offers the [CHOOSE EDITION] option and click it
+3.- Add the regular edition of the game to the cart
+4.- Open [https://www.paradoxinteractive.com/our-games/all-games]
+5.- Search for the same game and click [CHOOSE EDITION] again to select another edition</t>
+  </si>
+  <si>
+    <t>Navigate to the On Sale page</t>
+  </si>
+  <si>
+    <t>2. &amp; 4.- The On Sale page will open</t>
+  </si>
+  <si>
+    <t>2.- The games should display their sale tags in the upper-left corner of each card, showing the discount</t>
+  </si>
+  <si>
+    <t>Saving cart test</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
+2.- Add one or more games to the cart
+3.- Close the browser window, reopen it, and open [https://www.paradoxinteractive.com/our-games/cart]
+4.- Close the browser completely
+5.- Reopen the browser and go to [https://www.paradoxinteractive.com/our-games/cart]</t>
+  </si>
+  <si>
+    <t>2.- A pop-up should confirm each game as it is added, and the [🛒] button should show the number of games in the cart
+3. &amp; 5.- The cart page should open and display the latest saved information</t>
+  </si>
+  <si>
+    <t>2.- The game will be added to the cart, and a pop-up should confirm it has been added
+3.- The cart page should open
+4.- The [ADD PROMO CODE] button will appear below the input field
+     4.1.- A warning pop-up should appear next to the input field
+     4.2.- The input field will turn bold and red, and the message "Voucher has to be at least 8 characters long." will appear below it
+     4.3.- The entered code will disappear, and an error pop-up will appear in the bottom-right corner
+     4.4.- The discount will be applied, the summary will be updated with the discount information, and a confirmation pop-up will appear in the bottom-right corner</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
+2.- Add one game to the cart
+3.- Open the cart by clicking the [🛒] button
+4.- Remove the only game from the cart
+5.- Click [GO TO ALL GAMES]
+6.- Open the cart by clicking the [🛒] button
+7.- Click [← CONTINUE SHOPPING]</t>
+  </si>
+  <si>
+    <t>2.- A pop-up should confirm that the game has been added to the cart, and the [🛒] button should show the number of games in the cart
+3. &amp; 6.- The cart page should open
+4.- The game will be removed, and the cart will update to display the empty-cart state
+5. &amp; 7.- The All Games page should open</t>
   </si>
 </sst>
 </file>
@@ -512,25 +516,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79992065187536243"/>
+        <fgColor theme="9" tint="0.79989013336588644"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79992065187536243"/>
+        <fgColor theme="8" tint="0.79989013336588644"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79992065187536243"/>
+        <fgColor theme="5" tint="0.79989013336588644"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79992065187536243"/>
+        <fgColor theme="7" tint="0.79989013336588644"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -931,7 +935,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" style="4" customWidth="1"/>
@@ -989,458 +993,460 @@
         <v>11</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>64</v>
+        <v>12</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>66</v>
+        <v>14</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I2" s="12"/>
       <c r="J2" s="5"/>
     </row>
     <row r="3" spans="1:11" ht="255" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>67</v>
+        <v>19</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>106</v>
+        <v>21</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>69</v>
+        <v>22</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="3" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>13</v>
       </c>
       <c r="I4" s="5"/>
       <c r="J4" s="5"/>
     </row>
     <row r="5" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="J5" s="3"/>
     </row>
     <row r="6" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
     </row>
     <row r="7" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>76</v>
+        <v>47</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="135" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>80</v>
+        <v>52</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="J8" s="3"/>
       <c r="K8" s="13"/>
     </row>
     <row r="9" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>82</v>
+        <v>57</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
     </row>
     <row r="10" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C10" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>72</v>
-      </c>
       <c r="F10" s="3" t="s">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I10" s="3"/>
       <c r="J10" s="3" t="s">
-        <v>85</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
     </row>
     <row r="12" spans="1:11" ht="105" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>48</v>
+        <v>70</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>49</v>
+        <v>98</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>50</v>
+        <v>99</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
     </row>
     <row r="13" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
     </row>
     <row r="14" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>55</v>
+        <v>83</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>11</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>58</v>
+        <v>103</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I15" s="7"/>
       <c r="J15" s="7" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="165" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="180" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>59</v>
+        <v>86</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>61</v>
+        <v>104</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I16" s="3"/>
       <c r="J16" s="10"/>
     </row>
-    <row r="17" spans="1:10" s="9" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" s="9" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>63</v>
+        <v>92</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I17" s="8"/>
       <c r="J17" s="11"/>
     </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F18" s="13"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="C2:D3 C4:G4 C5:D16 E6:G6">
     <cfRule type="colorScale" priority="8">
       <colorScale>
@@ -1484,6 +1490,5 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>